<commit_message>
chore: arreglo 02 andres
</commit_message>
<xml_diff>
--- a/Tablas DB.xlsx
+++ b/Tablas DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3315783\GEAR EAGLE\Gear_eagle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FA6A18-0234-4D3E-915F-A093039A0F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2F13655-B5E7-4785-82B1-09C60B34641E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="705" firstSheet="8" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabla Cliente" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="180">
   <si>
     <t>id_cliente</t>
   </si>
@@ -577,6 +577,9 @@
   </si>
   <si>
     <t>cliente01@gmail.com</t>
+  </si>
+  <si>
+    <t>h</t>
   </si>
 </sst>
 </file>
@@ -1751,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" style="2" bestFit="1" customWidth="1"/>
@@ -1761,7 +1764,7 @@
     <col min="5" max="5" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1778,7 +1781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1795,7 +1798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1812,7 +1815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1829,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1846,7 +1849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1863,7 +1866,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1880,7 +1883,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1897,7 +1900,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1931,7 +1934,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1946,6 +1949,11 @@
       </c>
       <c r="E11" s="2">
         <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M15" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>